<commit_message>
Remove trailing space from the Open Item Analysis sheet name in the query workbook
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/resources/Open Closed Item details.xlsx
+++ b/backend/resources/Open Closed Item details.xlsx
@@ -5,16 +5,16 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amedeloitte-my.sharepoint.com/personal/vrashiwade_deloitte_com/Documents/Microsoft Teams Chat Files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amedeloitte-my.sharepoint.com/personal/ritwichatterjee_deloitte_com/Documents/Desktop/SAP Assessment Automation/backend/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="8_{F869414D-64A6-47F6-BE1D-F05B48CBD380}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BF616D90-0AB0-4473-8F58-C52007DC103A}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="8_{F869414D-64A6-47F6-BE1D-F05B48CBD380}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E4BA014C-7480-4B5A-A2CF-B0FFA6301AE0}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{4BE34D41-320F-4C26-94A0-9128AAD58B88}"/>
   </bookViews>
   <sheets>
     <sheet name="Year wise distribution" sheetId="1" r:id="rId1"/>
-    <sheet name="Open Item Analysis " sheetId="2" r:id="rId2"/>
+    <sheet name="Open Item Analysis" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -417,6 +417,18 @@
     <t xml:space="preserve">PERIO  </t>
   </si>
   <si>
+    <t>TECHNICAL</t>
+  </si>
+  <si>
+    <t>FINANCE</t>
+  </si>
+  <si>
+    <t>Material Management</t>
+  </si>
+  <si>
+    <t>Sales Documents</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <b/>
@@ -426,6 +438,484 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
+      <t>RL_TB:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+SELECT SUBSTRING(B.BDATU,1,4) AS Y,
+       SUBSTRING(B.BDATU,5,2) AS M,
+       SUM(CASE WHEN B.STATU = 'E' THEN 0 ELSE 1 END) AS OPEN_ENTRIES,
+       SUM(CASE WHEN B.STATU = 'E' THEN 1 ELSE 0 END) AS ELIGIBLE_FOR_ARCHIVING,
+       COUNT(*)                                       AS TOTAL_TRANSFER_REQS
+FROM LTBK B
+WHERE B.MANDT = '300'
+  AND B.BDATU &lt;&gt; '00000000'
+GROUP BY SUBSTRING(B.BDATU,1,4), SUBSTRING(B.BDATU,5,2)
+ORDER BY 1, 2;</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>RL_TA:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+SELECT SUBSTRING(A.BDATU,1,4) AS Y,
+       SUBSTRING(A.BDATU,5,2) AS M,
+       SUM(CASE WHEN A.KQUIT = 'X' THEN 0 ELSE 1 END) AS OPEN_ENTRIES,
+       SUM(CASE WHEN A.KQUIT = 'X' THEN 1 ELSE 0 END) AS ELIGIBLE_FOR_ARCHIVING,
+       COUNT(*)                                       AS TOTAL_TRANSFER_ORDERS
+FROM LTAK A
+WHERE A.MANDT = '300'
+  AND A.BDATU &lt;&gt; '00000000'
+GROUP BY SUBSTRING(A.BDATU,1,4), SUBSTRING(A.BDATU,5,2)
+ORDER BY 1, 2;</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>MM_INVBEL:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+SELECT SUBSTRING(K.BLDAT,1,4) AS Y,
+       SUBSTRING(K.BLDAT,5,2) AS M,
+       SUM(CASE WHEN S.IBLNR IS NOT NULL THEN 1 ELSE 0 END) AS OPEN_ENTRIES,
+       SUM(CASE WHEN S.IBLNR IS NULL     THEN 1 ELSE 0 END) AS ELIGIBLE_FOR_ARCHIVING,
+       COUNT(*)                                             AS TOTAL_INV_DOCS
+FROM IKPF K
+LEFT JOIN (SELECT DISTINCT MANDT, IBLNR, GJAHR
+           FROM ISEG
+           WHERE MANDT = '300'
+             AND XLOEK = ' '
+             AND XBUCH = ' ') S
+       ON  S.MANDT = K.MANDT
+       AND S.IBLNR = K.IBLNR
+       AND S.GJAHR = K.GJAHR
+WHERE K.MANDT = '300'
+  AND K.BLDAT &lt;&gt; '00000000'
+GROUP BY SUBSTRING(K.BLDAT,1,4), SUBSTRING(K.BLDAT,5,2)
+ORDER BY 1, 2;</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>RV_LIKP:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+SELECT SUBSTRING(L.ERDAT,1,4) AS Y,
+       SUBSTRING(L.ERDAT,5,2) AS M,
+       SUM(CASE WHEN V.WBSTK = 'C' AND V.FKSTK IN ('C',' ')
+                THEN 0
+                WHEN V.WBSTK IN ('A','B') OR V.FKSTK IN ('A','B')
+                THEN 1 ELSE 0 END)                           AS OPEN_ENTRIES,
+       SUM(CASE WHEN V.WBSTK = 'C' AND V.FKSTK IN ('C',' ')
+                THEN 1 ELSE 0 END)                           AS ELIGIBLE_FOR_ARCHIVING,
+       SUM(CASE WHEN V.WBSTK = 'C' AND V.FKSTK IN ('C',' ')
+                THEN 0
+                WHEN V.WBSTK IN ('A','B') OR V.FKSTK IN ('A','B')
+                THEN 0 ELSE 1 END)                           AS OTHER_REMAINING,
+       COUNT(*)                                              AS TOTAL_DELIVERIES
+FROM LIKP L
+INNER JOIN VBUK V
+        ON L.MANDT = V.MANDT
+       AND L.VBELN = V.VBELN
+WHERE L.MANDT = '300'
+  AND L.ERDAT &lt;&gt; '00000000'
+GROUP BY SUBSTRING(L.ERDAT,1,4), SUBSTRING(L.ERDAT,5,2)
+ORDER BY 1, 2;</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>MM_REBEL:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+ SELECT SUBSTRING(I.BUDAT,1,4) AS Y,
+       SUBSTRING(I.BUDAT,5,2) AS M,
+       SUM(CASE WHEN I.RBSTAT IN ('1','2','3','4','A','B','C')
+                THEN 1 ELSE 0 END)                           AS OPEN_ENTRIES,
+       SUM(CASE WHEN I.RBSTAT = '5'
+                THEN 1 ELSE 0 END)                           AS ELIGIBLE_FOR_ARCHIVING,
+       SUM(CASE WHEN I.RBSTAT NOT IN ('1','2','3','4','5','A','B','C')
+                THEN 1 ELSE 0 END)                           AS OTHER_REMAINING,
+       COUNT(*)                                              AS TOTAL_INVOICE_DOCS
+FROM RBKP I
+WHERE I.MANDT = '300'
+  AND I.BUDAT &lt;&gt; '00000000'
+GROUP BY SUBSTRING(I.BUDAT,1,4), SUBSTRING(I.BUDAT,5,2)
+ORDER BY 1, 2;</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SD_VTTK:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+SELECT SUBSTRING(T.ERDAT,1,4) AS Y,
+       SUBSTRING(T.ERDAT,5,2) AS M,
+       SUM(CASE WHEN T.STTRG BETWEEN '1' AND '6' THEN 1 ELSE 0 END) AS OPEN_ENTRIES,
+       SUM(CASE WHEN T.STTRG = '7' THEN 1 ELSE 0 END)               AS ELIGIBLE_FOR_ARCHIVING,
+       SUM(CASE WHEN T.STTRG NOT BETWEEN '1' AND '7' THEN 1 ELSE 0 END) AS OTHER_REMAINING,
+       COUNT(*)                                                     AS TOTAL_SHIPMENTS
+FROM VTTK T
+WHERE T.MANDT = '300'
+  AND T.ERDAT &lt;&gt; '00000000'
+GROUP BY SUBSTRING(T.ERDAT,1,4), SUBSTRING(T.ERDAT,5,2)
+ORDER BY 1, 2;</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>WORKITEM:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+SELECT SUBSTRING(W.WI_CD,1,4) AS Y,
+       SUBSTRING(W.WI_CD,5,2) AS M,
+       SUM(CASE WHEN W.WI_STAT IN ('READY','SELECTED','STARTED','COMMITTED','WAITING',
+                                   'ERROR','EXCPCAUGHT','EXCPHANDLR')
+                THEN 1 ELSE 0 END)                       AS OPEN_ENTRIES,
+       SUM(CASE WHEN W.WI_STAT IN ('COMPLETED','CANCELLED')
+                THEN 1 ELSE 0 END)                       AS ELIGIBLE_FOR_ARCHIVING,
+       SUM(CASE WHEN W.WI_STAT NOT IN ('READY','SELECTED','STARTED','COMMITTED','WAITING',
+                                       'ERROR','EXCPCAUGHT','EXCPHANDLR',
+                                       'COMPLETED','CANCELLED')
+                THEN 1 ELSE 0 END)                       AS OTHER_REMAINING,
+       COUNT(*)                                          AS TOTAL_WORK_ITEMS
+FROM SWWWIHEAD W
+WHERE W.MANDT = '300'
+  AND W.WI_CD &lt;&gt; '00000000'
+GROUP BY SUBSTRING(W.WI_CD,1,4), SUBSTRING(W.WI_CD,5,2)
+ORDER BY 1, 2;</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>MM_EBAN:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+SELECT SUBSTRING(R.BADAT,1,4) AS Y,
+       SUBSTRING(R.BADAT,5,2) AS M,
+       SUM(CASE WHEN R.LOEKZ &lt;&gt; ' ' OR R.EBAKZ = 'X'
+                THEN 0 ELSE 1 END)                AS OPEN_ENTRIES,
+       SUM(CASE WHEN R.LOEKZ &lt;&gt; ' ' OR R.EBAKZ = 'X'
+                THEN 1 ELSE 0 END)                AS ELIGIBLE_FOR_ARCHIVING,
+       COUNT(*)                                   AS TOTAL_REQ_ITEMS
+FROM EBAN R
+WHERE R.MANDT = '300'
+  AND R.BADAT &lt;&gt; '00000000'
+GROUP BY SUBSTRING(R.BADAT,1,4), SUBSTRING(R.BADAT,5,2)
+ORDER BY 1, 2;</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">SD_VBRK: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+SELECT Y,
+       M,
+       SUM(CASE WHEN CAT = 'O' THEN 1 ELSE 0 END) AS OPEN_ENTRIES,
+       SUM(CASE WHEN CAT = 'E' THEN 1 ELSE 0 END) AS ELIGIBLE_FOR_ARCHIVING,
+       SUM(CASE WHEN CAT = 'R' THEN 1 ELSE 0 END) AS OTHER_REMAINING,
+       COUNT(*)                                   AS TOTAL_BILLING_DOCS
+FROM (
+    SELECT SUBSTRING(B.FKDAT,1,4) AS Y,
+           SUBSTRING(B.FKDAT,5,2) AS M,
+           CASE WHEN B.RFBSK IN ('A','B','E','F','G')
+                  OR EXISTS (SELECT 1 FROM BSID D
+                             WHERE D.MANDT = B.MANDT
+                               AND D.BUKRS = B.BUKRS
+                               AND D.BELNR = B.BELNR
+                               AND D.GJAHR = B.GJAHR)
+                THEN 'O'
+                WHEN B.RFBSK = 'C' THEN 'E'
+                ELSE 'R'
+           END AS CAT
+    FROM VBRK B
+    WHERE B.MANDT = '300' AND B.FKDAT &lt;&gt; '00000000'
+) T
+GROUP BY Y, M
+ORDER BY Y, M;</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>IDOC:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+SELECT Y,
+       M,
+       SUM(CASE WHEN CAT = 'O' THEN 1 ELSE 0 END) AS OPEN_ENTRIES,
+       SUM(CASE WHEN CAT = 'E' THEN 1 ELSE 0 END) AS ELIGIBLE_FOR_ARCHIVING,
+       SUM(CASE WHEN CAT = 'R' THEN 1 ELSE 0 END) AS OTHER_REMAINING,
+       COUNT(*)                                   AS TOTAL_IDOCS
+FROM (
+    SELECT SUBSTRING(I.CREDAT,1,4) AS Y,
+           SUBSTRING(I.CREDAT,5,2) AS M,
+           CASE WHEN I.STATUS IN ('12','31','41','53','68') THEN 'E'
+                WHEN I.STATUS IN ('02','03','30','51','56','64','66') THEN 'O'
+                ELSE 'R' END AS CAT
+    FROM EDIDC I
+    WHERE I.MANDT = '300' AND I.CREDAT &lt;&gt; '00000000'
+) T
+GROUP BY Y, M
+ORDER BY Y, M;</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>FI_DOCUMNT:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+SELECT Y,
+       M,
+       SUM(CASE WHEN CAT = 'O' THEN 1 ELSE 0 END) AS OPEN_ENTRIES,
+       SUM(CASE WHEN CAT = 'E' THEN 1 ELSE 0 END) AS ELIGIBLE_FOR_ARCHIVING,
+       COUNT(*)                                   AS TOTAL_DOCS
+FROM (
+    SELECT SUBSTRING(B.BUDAT,1,4) AS Y,
+           SUBSTRING(B.BUDAT,5,2) AS M,
+           CASE WHEN B.BSTAT &lt;&gt; ' '
+                  OR EXISTS (SELECT 1 FROM BSID D
+                             WHERE D.MANDT = B.MANDT AND D.BUKRS = B.BUKRS
+                               AND D.BELNR = B.BELNR AND D.GJAHR = B.GJAHR)
+                  OR EXISTS (SELECT 1 FROM BSIK K
+                             WHERE K.MANDT = B.MANDT AND K.BUKRS = B.BUKRS
+                               AND K.BELNR = B.BELNR AND K.GJAHR = B.GJAHR)
+                  OR EXISTS (SELECT 1 FROM BSIS S
+                             WHERE S.MANDT = B.MANDT AND S.BUKRS = B.BUKRS
+                               AND S.BELNR = B.BELNR AND S.GJAHR = B.GJAHR
+                               AND S.XOPVW = 'X')
+                THEN 'O' ELSE 'E'
+           END AS CAT
+    FROM BKPF B
+    WHERE B.MANDT = '300' AND B.BUDAT &lt;&gt; '00000000'
+) T
+GROUP BY Y, M
+ORDER BY Y, M;</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>MM_EKKO:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+ SELECT SUBSTRING(H.AEDAT,1,4) AS Y, SUBSTRING(H.AEDAT,5,2) AS SELECT Y,
+       M,
+       SUM(CASE WHEN CAT = 'O' THEN 1 ELSE 0 END) AS OPEN_ENTRIES,
+       SUM(CASE WHEN CAT = 'E' THEN 1 ELSE 0 END) AS ELIGIBLE_FOR_ARCHIVING,
+       COUNT(*)                                   AS TOTAL_DOCS
+FROM (
+    SELECT SUBSTRING(H.AEDAT,1,4) AS Y,
+           SUBSTRING(H.AEDAT,5,2) AS M,
+           CASE WHEN EXISTS (SELECT 1 FROM EKPO P
+                             WHERE P.MANDT = H.MANDT
+                               AND P.EBELN = H.EBELN
+                               AND P.LOEKZ = ' '
+                               AND ((P.ELIKZ = ' ' AND P.WEPOS = 'X')
+                                 OR (P.EREKZ = ' ' AND P.REPOS = 'X')))
+                THEN 'O'
+                ELSE 'E'
+           END AS CAT
+    FROM EKKO H
+    WHERE H.MANDT = '300' AND H.AEDAT &lt;&gt; '00000000'
+) T
+GROUP BY Y, M
+ORDER BY Y, M;</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>SD_VBAK:</t>
     </r>
     <r>
@@ -437,13 +927,24 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">
-SELECT SUBSTRING(K.ERDAT,1,4) AS Y, SUBSTRING(K.ERDAT,5,2) AS M,
-       CASE WHEN V.ABSTK = 'C' OR V.GBSTK = 'C' THEN 'E'
-            WHEN V.GBSTK IN ('A','B') THEN 'O'
-            ELSE 'R' END AS CAT
-FROM VBAK K
-INNER JOIN VBUK V ON K.MANDT = V.MANDT AND K.VBELN = V.VBELN
-WHERE K.MANDT = '300' AND K.ERDAT &lt;&gt; '00000000'</t>
+SELECT Y,
+       M,
+       SUM(CASE WHEN CAT = 'O' THEN 1 ELSE 0 END) AS OPEN_ENTRIES,
+       SUM(CASE WHEN CAT = 'E' THEN 1 ELSE 0 END) AS ELIGIBLE_FOR_ARCHIVING,
+       SUM(CASE WHEN CAT = 'R' THEN 1 ELSE 0 END) AS OTHER_REMAINING,
+       COUNT(*)                                   AS TOTAL_DOCS
+FROM (
+    SELECT SUBSTRING(K.ERDAT,1,4) AS Y,
+           SUBSTRING(K.ERDAT,5,2) AS M,
+           CASE WHEN V.ABSTK = 'C' OR V.GBSTK = 'C' THEN 'E'
+                WHEN V.GBSTK IN ('A','B') THEN 'O'
+                ELSE 'R' END AS CAT
+    FROM VBAK K
+    INNER JOIN VBUK V ON K.MANDT = V.MANDT AND K.VBELN = V.VBELN
+    WHERE K.MANDT = '300' AND K.ERDAT &lt;&gt; '00000000'
+) T
+GROUP BY Y, M
+ORDER BY Y, M;</t>
     </r>
   </si>
   <si>
@@ -456,7 +957,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">SD_VBRK: </t>
+      <t>BC_SBAL:</t>
     </r>
     <r>
       <rPr>
@@ -467,360 +968,21 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">
-SELECT SUBSTRING(B.FKDAT,1,4) AS Y, SUBSTRING(B.FKDAT,5,2) AS M,
-       CASE WHEN B.RFBSK IN ('A','B','E','F','G')
-              OR EXISTS (SELECT 1 FROM BSID D WHERE D.MANDT = B.MANDT
-                         AND D.BUKRS = B.BUKRS AND D.BELNR = B.BELNR AND D.GJAHR = B.GJAHR)
-                 THEN 'O'
-            WHEN B.RFBSK = 'C' THEN 'E'
-            ELSE 'R' END AS CAT
-FROM VBRK B
-WHERE B.MANDT = '300' AND B.FKDAT &lt;&gt; '00000000'</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>SD_VTTK:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-SELECT SUBSTRING(T.ERDAT,1,4) AS Y, SUBSTRING(T.ERDAT,5,2) AS M,
-       CASE WHEN T.STTRG = '7' THEN 'E'
-            WHEN T.STTRG BETWEEN '1' AND '6' THEN 'O'
-            ELSE 'R' END AS CAT
-FROM VTTK T
-WHERE T.MANDT = '300' AND T.ERDAT &lt;&gt; '00000000'</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>RV_LIKP:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-SELECT SUBSTRING(L.ERDAT,1,4) AS Y, SUBSTRING(L.ERDAT,5,2) AS M,
-       CASE WHEN V.WBSTK = 'C' AND V.FKSTK IN ('C',' ') THEN 'E'
-            WHEN V.WBSTK IN ('A','B') OR V.FKSTK IN ('A','B') THEN 'O'
-            ELSE 'R' END AS CAT
-FROM LIKP L
-INNER JOIN VBUK V ON L.MANDT = V.MANDT AND L.VBELN = V.VBELN
-WHERE L.MANDT = '300' AND L.ERDAT &lt;&gt; '00000000'</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>MM_EKKO:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
- SELECT SUBSTRING(H.AEDAT,1,4) AS Y, SUBSTRING(H.AEDAT,5,2) AS M,
-       CASE WHEN EXISTS (SELECT 1 FROM EKPO P
-                         WHERE P.MANDT = H.MANDT AND P.EBELN = H.EBELN AND P.LOEKZ = ' '
-                           AND ((P.ELIKZ = ' ' AND P.WEPOS = 'X')
-                             OR (P.EREKZ = ' ' AND P.REPOS = 'X')))
-                 THEN 'O'
-            ELSE 'E' END AS CAT
-FROM EKKO H
-WHERE H.MANDT = '300' AND H.AEDAT &lt;&gt; '00000000'</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>MM_EBAN:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-SELECT SUBSTRING(R.BADAT,1,4) AS Y, SUBSTRING(R.BADAT,5,2) AS M,
-       CASE WHEN R.LOEKZ &lt;&gt; ' ' OR R.EBAKZ = 'X' THEN 'E' ELSE 'O' END AS CAT
-FROM EBAN R
-WHERE R.MANDT = '300' AND R.BADAT &lt;&gt; '00000000'</t>
-    </r>
-  </si>
-  <si>
-    <t>MM_REBEL:
- SELECT SUBSTRING(I.BUDAT,1,4) AS Y, SUBSTRING(I.BUDAT,5,2) AS M,
-       CASE WHEN I.RBSTAT = '5' THEN 'E'
-            WHEN I.RBSTAT IN ('1','2','3','4','A','B','C') THEN 'O'
-            ELSE 'R' END AS CAT
-FROM RBKP I
-WHERE I.MANDT = '300' AND I.BUDAT &lt;&gt; '00000000'</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>MM_INVBEL:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-SELECT SUBSTRING(K.BLDAT,1,4) AS Y, SUBSTRING(K.BLDAT,5,2) AS M,
-       CASE WHEN EXISTS (SELECT 1 FROM ISEG S
-                         WHERE S.MANDT = K.MANDT AND S.IBLNR = K.IBLNR AND S.GJAHR = K.GJAHR
-                           AND S.XLOEK = ' ' AND S.XBUCH = ' ')
-                 THEN 'O' ELSE 'E' END AS CAT
-FROM IKPF K
-WHERE K.MANDT = '300' AND K.BLDAT &lt;&gt; '00000000'</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>RL_TA:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-SELECT SUBSTRING(A.BDATU,1,4) AS Y, SUBSTRING(A.BDATU,5,2) AS M,
-       CASE WHEN A.KQUIT = 'X' THEN 'E' ELSE 'O' END AS CAT
-FROM LTAK A
-WHERE A.MANDT = '300' AND A.BDATU &lt;&gt; '00000000'</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>RL_TB:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-SELECT SUBSTRING(B.BDATU,1,4) AS Y, SUBSTRING(B.BDATU,5,2) AS M,
-       CASE WHEN B.STATU = 'E' THEN 'E' ELSE 'O' END AS CAT
-FROM LTBK B
-WHERE B.MANDT = '300' AND B.BDATU &lt;&gt; '00000000'</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>FI_DOCUMNT:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-SELECT SUBSTRING(B.BUDAT,1,4) AS Y, SUBSTRING(B.BUDAT,5,2) AS M,
-       CASE WHEN B.BSTAT &lt;&gt; ' '
-              OR EXISTS (SELECT 1 FROM BSID D WHERE D.MANDT = B.MANDT AND D.BUKRS = B.BUKRS
-                         AND D.BELNR = B.BELNR AND D.GJAHR = B.GJAHR)
-              OR EXISTS (SELECT 1 FROM BSIK K WHERE K.MANDT = B.MANDT AND K.BUKRS = B.BUKRS
-                         AND K.BELNR = B.BELNR AND K.GJAHR = B.GJAHR)
-              OR EXISTS (SELECT 1 FROM BSIS S WHERE S.MANDT = B.MANDT AND S.BUKRS = B.BUKRS
-                         AND S.BELNR = B.BELNR AND S.GJAHR = B.GJAHR AND S.XOPVW = 'X')
-                 THEN 'O' ELSE 'E' END AS CAT
-FROM BKPF B
-WHERE B.MANDT = '300' AND B.BUDAT &lt;&gt; '00000000'</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>IDOC:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-SELECT SUBSTRING(I.CREDAT,1,4) AS Y, SUBSTRING(I.CREDAT,5,2) AS M,
-       CASE WHEN I.STATUS IN ('12','31','41','53','68') THEN 'E'
-            WHEN I.STATUS IN ('02','03','30','51','56','64','66') THEN 'O'
-            ELSE 'R' END AS CAT
-FROM EDIDC I
-WHERE I.MANDT = '300' AND I.CREDAT &lt;&gt; '00000000'</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>WORKITEM:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-SELECT SUBSTRING(W.WI_CD,1,4) AS Y, SUBSTRING(W.WI_CD,5,2) AS M,
-       CASE WHEN W.WI_STAT IN ('COMPLETED','CANCELLED') THEN 'E'
-            WHEN W.WI_STAT IN ('READY','SELECTED','STARTED','COMMITTED','WAITING','ERROR',
-                               'EXCPCAUGHT','EXCPHANDLR') THEN 'O'
-            ELSE 'R' END AS CAT
-FROM SWWWIHEAD W
-WHERE W.MANDT = '300' AND W.WI_CD &lt;&gt; '00000000'</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>BC_SBAL:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-SELECT SUBSTRING(L.ALDATE,1,4) AS Y, SUBSTRING(L.ALDATE,5,2) AS M,
-       CASE WHEN L.DEL_BEFORE = 'X' AND L.ALDATE_DEL &gt;= TO_VARCHAR(CURRENT_DATE,'YYYYMMDD')
-                 THEN 'O' ELSE 'E' END AS CAT
+SELECT SUBSTRING(L.ALDATE,1,4) AS Y,
+       SUBSTRING(L.ALDATE,5,2) AS M,
+       SUM(CASE WHEN L.DEL_BEFORE = 'X'
+                 AND L.ALDATE_DEL &gt;= TO_VARCHAR(CURRENT_DATE,'YYYYMMDD')
+                THEN 1 ELSE 0 END)                           AS OPEN_ENTRIES,
+       SUM(CASE WHEN L.DEL_BEFORE = 'X'
+                 AND L.ALDATE_DEL &gt;= TO_VARCHAR(CURRENT_DATE,'YYYYMMDD')
+                THEN 0 ELSE 1 END)                           AS ELIGIBLE_FOR_ARCHIVING,
+       COUNT(*)                                              AS TOTAL_LOG_HEADERS
 FROM BALHDR L
-WHERE L.MANDT = '300' AND L.ALDATE &lt;&gt; '00000000'</t>
-    </r>
-  </si>
-  <si>
-    <t>TECHNICAL</t>
-  </si>
-  <si>
-    <t>FINANCE</t>
-  </si>
-  <si>
-    <t>Material Management</t>
-  </si>
-  <si>
-    <t>Sales Documents</t>
+WHERE L.MANDANT = '300'
+  AND L.ALDATE &lt;&gt; '00000000'
+GROUP BY SUBSTRING(L.ALDATE,1,4), SUBSTRING(L.ALDATE,5,2)
+ORDER BY 1, 2;</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -1806,7 +1968,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F99CBC0C-AC41-4D3B-8D5C-2DAE2BAE254D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{126C7324-5A2B-461D-B090-784B2DF5FDF3}">
   <dimension ref="B1:H13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1818,30 +1980,30 @@
   <sheetData>
     <row r="1" spans="2:8" s="6" customFormat="1" ht="21" x14ac:dyDescent="0.35">
       <c r="B1" s="9" t="s">
-        <v>142</v>
+        <v>128</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>141</v>
+        <v>127</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>140</v>
+        <v>126</v>
       </c>
       <c r="H1" s="9" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
     </row>
     <row r="2" spans="2:8" ht="223.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="7" t="s">
-        <v>125</v>
+        <v>141</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="H2" s="7" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.35">
@@ -1852,13 +2014,13 @@
     </row>
     <row r="4" spans="2:8" ht="235" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B4" s="7" t="s">
-        <v>126</v>
+        <v>137</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.35">
@@ -1866,15 +2028,15 @@
       <c r="D5" s="12"/>
       <c r="H5" s="11"/>
     </row>
-    <row r="6" spans="2:8" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:8" ht="299.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>131</v>
+        <v>134</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>133</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.35">
@@ -1882,32 +2044,32 @@
       <c r="D7" s="12"/>
       <c r="H7" s="11"/>
     </row>
-    <row r="8" spans="2:8" ht="141" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:8" ht="354" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="7" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B9" s="11"/>
       <c r="D9" s="12"/>
     </row>
-    <row r="10" spans="2:8" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:8" ht="204.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="5"/>
       <c r="D10" s="8" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B11" s="5"/>
       <c r="D11" s="12"/>
     </row>
-    <row r="12" spans="2:8" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:8" ht="217.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B12" s="5"/>
       <c r="D12" s="8" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.35">

</xml_diff>